<commit_message>
Logins, Events tab, imports that read their own dates, faster reads
- Handed-out logins (AUTH_ACCOUNTS): signed session cookie, login page, projects owned by the account that made them (migration 0008); the Audit screen is gone.
- Events tab lists community events and closures with their berths.
- Uploading a workbook with no "planning until" takes the import window from the file's own dates, and commit moves the project's today to the window start when it falls outside. No more "0 bookings" on a decades-old file.
- Vessels: All / Length known / Length unknown filter; search and filter run in memory on the one fetched list.
- Berths lose `kind` (migration 0007): every row is exclusive and a missing length means "fit unverified".
- Reads reuse the project row loaded for authorization (one Neon round trip less per request); the Conflicts list keeps its rows while a filter loads.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/dock-template.xlsx
+++ b/public/dock-template.xlsx
@@ -28,18 +28,11 @@
     <comment ref="B1" authorId="0">
       <text>
         <r>
-          <t>berth = one occupant at a time; section = shared area</t>
+          <t>Leave blank if it isn't on record — nothing booked there can be checked for fit</t>
         </r>
       </text>
     </comment>
     <comment ref="C1" authorId="0">
-      <text>
-        <r>
-          <t>Required for a berth, blank for a section</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0">
       <text>
         <r>
           <t>Optional row order</t>
@@ -148,14 +141,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t>Name</t>
   </si>
   <si>
-    <t>Kind</t>
-  </si>
-  <si>
     <t>Length (ft)</t>
   </si>
   <si>
@@ -163,9 +153,6 @@
   </si>
   <si>
     <t>e.g. North Pier West</t>
-  </si>
-  <si>
-    <t>berth</t>
   </si>
   <si>
     <t>Draft (ft)</t>
@@ -602,16 +589,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D500"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -621,531 +607,19 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="B2" s="2">
+        <v>410</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2">
-        <v>410</v>
-      </c>
-      <c r="D2" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="202" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="203" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="204" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="205" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="206" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="207" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="208" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="210" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="211" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="212" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="213" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="214" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="215" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="216" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="217" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="218" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="219" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="220" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="221" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="224" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="225" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="227" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="240" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="241" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="243" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="244" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="245" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="246" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="247" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="248" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="249" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="250" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="251" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="252" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="253" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="254" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="255" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="256" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="257" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="258" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="259" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="260" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="261" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="262" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="263" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="264" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="265" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="266" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="267" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="268" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="269" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="270" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="271" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="272" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="273" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="274" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="275" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="276" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="277" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="278" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="279" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="280" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="281" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="282" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="283" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="284" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="285" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="286" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="287" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="288" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="289" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="290" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="291" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="292" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="293" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="294" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="295" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="296" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="297" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="298" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="299" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="300" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="301" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="302" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="303" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="304" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="305" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="306" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="307" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="308" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="309" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="310" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="311" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="312" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="313" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="314" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="315" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="316" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="317" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="318" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="319" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="320" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="321" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="322" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="323" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="324" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="325" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="326" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="327" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="328" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="329" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="330" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="331" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="332" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="333" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="334" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="335" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="336" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="337" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="338" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="339" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="340" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="341" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="342" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="343" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="344" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="345" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="346" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="347" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="348" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="349" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="350" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="351" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="352" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="353" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="354" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="355" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="356" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="357" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="358" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="359" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="360" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="361" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="362" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="363" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="364" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="365" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="366" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="367" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="368" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="369" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="370" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="371" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="372" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="373" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="374" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="375" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="376" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="377" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="378" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="379" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="380" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="381" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="382" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="383" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="384" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="385" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="386" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="387" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="388" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="389" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="390" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="391" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="392" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="393" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="394" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="395" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="396" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="397" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="398" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="399" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="400" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="401" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="402" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="403" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="404" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="405" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="406" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="407" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="408" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="409" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="410" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="411" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="412" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="413" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="414" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="415" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="416" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="417" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="418" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="419" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="420" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="421" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="422" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="423" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="424" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="425" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="426" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="427" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="428" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="429" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="430" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="431" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="432" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="433" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="434" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="435" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="436" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="437" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="438" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="439" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="440" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="441" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="442" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="443" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="444" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="445" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="446" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="447" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="448" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="449" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="450" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="451" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="452" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="453" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="454" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="455" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="456" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="457" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="458" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="459" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="460" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="461" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="462" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="463" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="464" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="465" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="466" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="467" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="468" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="469" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="470" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="471" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="472" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="473" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="474" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="475" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="476" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="477" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="478" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="479" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="480" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="481" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="482" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="483" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="484" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="485" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="486" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="487" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="488" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="489" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="490" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="491" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="492" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="493" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="494" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="495" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="496" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="497" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="498" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="499" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="500" spans="2:2" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Not allowed" error="Use one of: berth, section" sqref="B10:B500">
-      <formula1>"berth,section"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Not allowed" error="Use one of: berth, section" sqref="B2:B500">
-      <formula1>"berth,section"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <legacyDrawing r:id="rId2"/>
@@ -1169,21 +643,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2">
         <v>120</v>
@@ -1192,10 +666,10 @@
         <v>9.5</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1219,33 +693,33 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D2" s="5">
         <v>46451</v>
@@ -1254,7 +728,7 @@
         <v>46455</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25"/>

</xml_diff>